<commit_message>
feat: Add AI integration tests and enhance documentation for compliance and extraction prompts
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -713,70 +713,287 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="10" t="inlineStr"/>
@@ -941,7 +1158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -987,76 +1204,334 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1266,34 +1741,132 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="10" t="inlineStr"/>
@@ -1543,46 +2116,186 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="10" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: Enhance validation engine to save workbook in place and log the action; add test for workbook submission
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -526,7 +526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -667,8 +667,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -996,10 +996,1419 @@
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1017,7 +2426,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1158,8 +2567,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D81"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1525,6 +2934,1656 @@
         </is>
       </c>
       <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -1549,7 +4608,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1695,8 +4754,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1869,46 +4928,644 @@
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1926,7 +5583,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -2070,8 +5727,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -2298,34 +5955,914 @@
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
feat: Enhance health checks for cloud providers and local model; refactor startup validation and logging events
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2402,6 +2402,855 @@
         </is>
       </c>
       <c r="D69" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Alice Nguyen  |  Room: 5A
@@ -2567,7 +3416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4584,6 +5433,996 @@
         </is>
       </c>
       <c r="D81" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -4754,7 +6593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5558,6 +7397,390 @@
         </is>
       </c>
       <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
 Resident: Edna Kowalski  |  Room: 2B
@@ -5727,7 +7950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6864,6 +9087,552 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
feat: Update environment configuration for local model auto-download; enhance startup validation logging and apply environment variables
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3251,6 +3251,1138 @@
         </is>
       </c>
       <c r="D102" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Alice Nguyen  |  Room: 5A
@@ -3416,7 +4548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:D172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6423,6 +7555,1326 @@
         </is>
       </c>
       <c r="D120" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -6593,7 +9045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7781,6 +10233,518 @@
         </is>
       </c>
       <c r="D48" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
 Resident: Edna Kowalski  |  Room: 2B
@@ -7950,7 +10914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9633,6 +12597,734 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
feat: Enhance health checks and logging for AI providers; add diagnostics and update model download logging
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D146"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4383,6 +4383,855 @@
         </is>
       </c>
       <c r="D146" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Alice Nguyen  |  Room: 5A
@@ -4548,7 +5397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D172"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8875,6 +9724,996 @@
         </is>
       </c>
       <c r="D172" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
         <is>
           <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -9045,7 +10884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10745,6 +12584,390 @@
         </is>
       </c>
       <c r="D68" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
         <is>
           <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
 Resident: Edna Kowalski  |  Room: 2B
@@ -10914,7 +13137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13325,6 +15548,552 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
feat: Enhance documentation and logging throughout the codebase; improve model loading, health checks, and error handling
</commit_message>
<xml_diff>
--- a/data/raw/Your_Output_File.xlsx
+++ b/data/raw/Your_Output_File.xlsx
@@ -526,7 +526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -667,8 +667,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -713,76 +713,1136 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_VITALS. Trigger Condition: Missing vital sign components: BP, RR, Temperature, SpO2.. Evidence Found: Progress Note — Fall Incident
+Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
+Date: 10 June 2025  |  Time of fall: 08:05
+Resident found on floor near wardrobe in her room during morning round. Not witnessed. Com. Missing Requirement: Policy requires a full set of observations on Day 1.. Recommendation: Record a full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 11 June 2025
+Alice slept well. Back pain seems a bit better today. Up and moving around.
+Vitals: BP 136/80, HR 74, RR 15, Temp 36.4, SpO2 98%.
+No new symptoms no. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Alice Nguyen  |  Room: 5A
+Date: 12 June 2025
+Alice in good spirits. Joined group activity this morning. Son visited yesterday.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -800,7 +1860,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -941,8 +2001,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -987,76 +2047,1324 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Witnessed status</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_FALL_DETAILS. Trigger Condition: Whether the fall was witnessed was not documented.. Evidence Found: Progress Note — Fall Incident
+Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
+Date: 10 June 2025  |  Time of fall: 11:20
+Resident found on floor in bathroom. Complaining of right shoulder pain — rates 6/10. Sma. Missing Requirement: Policy requires the incident details to be documented on Day 1.. Recommendation: State whether the fall was witnessed or unwitnessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Pain status</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Current pain status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether pain improved, worsened, or resolved using the 0-10 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Weight-bearing status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Vital signs</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: No full set of observations was recorded.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Record at least one full set of observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 11 June 2025
+Robert rested well overnight. Shoulder still sore but managing. X-ray result came back — no fracture, soft tissue injury only. Dr Nasseri informed.
+. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Robert Singh  |  Room: 11C
+Date: 12 June 2025
+Robert doing well. Shoulder much better. Daughter visited last night.. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1074,7 +3382,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1220,8 +3528,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1266,76 +3574,516 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Falls risk score</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ACTIONS. Trigger Condition: Falls risk score was not reassessed.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires the full follow-up documentation for Day 1.. Recommendation: Record the reassessed falls risk score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pain scale</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D1_ASSESSMENT. Trigger Condition: Pain level was not recorded on the required 0-10 scale.. Evidence Found: Progress Note — Fall Incident
+Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
+Date: 10 June 2025  |  Time of fall: 16:45
+Resident witnessed falling near the nurses station by RN James Obi. Resident complains of. Missing Requirement: Policy requires a documented initial condition assessment.. Recommendation: Document pain using a 0-10 numeric scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Vague</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mobility status</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Mobility status is not explicit enough.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: State clearly whether the resident can full weight-bear without pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GP follow-up</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: GP follow-up was not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any Day 1 GP advice was actioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Care plan changes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: Care plan changes were not documented.. Evidence Found: Progress Note
+Resident: Edna Kowalski  |  Room: 2B
+Date: 11 June 2025
+Left ankle swelling has reduced slightly overnight. Pain rates 3/10 this morning — improvement from yesterday.
+Mobilising with some caution but able. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document any changes to the care plan since Day 1.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1353,7 +4101,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1497,8 +4245,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1543,76 +4291,732 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>New symptoms</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Policy Rule: D2_UPDATE. Trigger Condition: New symptoms since Day 1 were not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 11 June 2025
+Left knee pain improved — rates 2/10 this morning. Resident mobilising well with walking stick. Full weight-bearing confirmed.
+Vitals: BP 140/86, H. Missing Requirement: Policy requires continuation documentation on Day 2.. Recommendation: Document whether any new symptoms appeared since Day 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pain outcome</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Pain outcome was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document whether pain has resolved or remains ongoing with an escalation plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mobility baseline</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Mobility baseline was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Confirm whether mobility has returned to baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Outstanding actions</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Outstanding actions were not resolved or documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the resolution of any outstanding actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Incident closure</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The incident was not formally closed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document that the post-fall monitoring period is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Prevention plan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: The falls prevention plan was not reviewed.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Document the updated falls prevention plan review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Escalation</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Policy Rule: D3_CLOSE. Trigger Condition: Escalation status was not documented.. Evidence Found: Progress Note
+Resident: Thomas Brennan  |  Room: 9F
+Date: 12 June 2025
+Thomas feeling well today. Knee pain has settled — rates 0/10. Mobilising independently with walking stick, no concerns.
+Wife visited again this af. Missing Requirement: Policy requires closure or escalation documentation on Day 3.. Recommendation: Escalate if the resident has not stabilised, or document why escalation is not needed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>